<commit_message>
Update tariffs from refreshed table and implement advanced carrier allocation rules (Олимп, Агро-Авто, Наткар, Примум, Азимут, Буш-Авто)
</commit_message>
<xml_diff>
--- a/ТАРИФЫ РК ТАБЛИЦА.xlsx
+++ b/ТАРИФЫ РК ТАБЛИЦА.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stanislavhvostov/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49752AAE-2B12-1B45-95A5-D8CB7CA17993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{232C4FC2-3123-E84D-8522-44CDF2B353B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="580" windowWidth="27040" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1373,9 +1373,7 @@
         <v>48800</v>
       </c>
       <c r="G6" s="14"/>
-      <c r="H6" s="14">
-        <v>65000</v>
-      </c>
+      <c r="H6" s="14"/>
       <c r="I6" s="14"/>
       <c r="J6" s="14">
         <v>56500</v>
@@ -1389,7 +1387,7 @@
       <c r="M6" s="14"/>
       <c r="N6" s="45">
         <f t="shared" ref="N6:N22" si="0">AVERAGE(B6:M6)</f>
-        <v>59383.333333333336</v>
+        <v>58260</v>
       </c>
       <c r="P6" s="2" t="s">
         <v>6</v>
@@ -1413,9 +1411,7 @@
         <v>57950</v>
       </c>
       <c r="G7" s="14"/>
-      <c r="H7" s="14">
-        <v>70000</v>
-      </c>
+      <c r="H7" s="14"/>
       <c r="I7" s="14"/>
       <c r="J7" s="14">
         <v>65000</v>
@@ -1429,7 +1425,7 @@
       <c r="M7" s="14"/>
       <c r="N7" s="45">
         <f t="shared" si="0"/>
-        <v>67991.666666666672</v>
+        <v>67590</v>
       </c>
       <c r="P7" s="2" t="s">
         <v>7</v>
@@ -1499,9 +1495,7 @@
       <c r="G9" s="14">
         <v>118320</v>
       </c>
-      <c r="H9" s="14">
-        <v>128000</v>
-      </c>
+      <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14">
         <v>133800</v>
@@ -1517,7 +1511,7 @@
       </c>
       <c r="N9" s="45">
         <f t="shared" si="0"/>
-        <v>137733.70000000001</v>
+        <v>138815.22222222222</v>
       </c>
       <c r="P9" s="2" t="s">
         <v>9</v>
@@ -1581,9 +1575,7 @@
         <v>177917</v>
       </c>
       <c r="G11" s="14"/>
-      <c r="H11" s="14">
-        <v>175000</v>
-      </c>
+      <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14">
         <v>180000</v>
@@ -1599,7 +1591,7 @@
       </c>
       <c r="N11" s="45">
         <f t="shared" si="0"/>
-        <v>205613</v>
+        <v>209439.625</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>11</v>
@@ -3665,18 +3657,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D8 J8 F8 H8">
-    <cfRule type="colorScale" priority="329">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D8">
     <cfRule type="colorScale" priority="347">
       <colorScale>
@@ -3725,6 +3705,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D12 J12 F12 H12">
+    <cfRule type="colorScale" priority="325">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D12">
     <cfRule type="colorScale" priority="343">
       <colorScale>
@@ -3749,18 +3741,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D14 J14 F14 H14">
-    <cfRule type="colorScale" priority="323">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D14">
     <cfRule type="colorScale" priority="341">
       <colorScale>
@@ -3785,18 +3765,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D16 J16 F16 H16">
-    <cfRule type="colorScale" priority="321">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D16">
     <cfRule type="colorScale" priority="339">
       <colorScale>
@@ -3845,18 +3813,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D22 J22 F22 H22">
-    <cfRule type="colorScale" priority="315">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D22">
     <cfRule type="colorScale" priority="333">
       <colorScale>
@@ -3917,68 +3873,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5 J5 D5 H5">
-    <cfRule type="colorScale" priority="332">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F6 J6 D6 H6">
-    <cfRule type="colorScale" priority="331">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7 J7 D7 H7">
-    <cfRule type="colorScale" priority="330">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F9 J9 D9 H9">
-    <cfRule type="colorScale" priority="328">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F10 J10 D10 H10">
-    <cfRule type="colorScale" priority="327">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F13 J13 D13 H13">
-    <cfRule type="colorScale" priority="324">
+  <conditionalFormatting sqref="F11 J11 D11 H11">
+    <cfRule type="colorScale" priority="326">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4397,32 +4293,32 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H17 J17 D17 F17">
-    <cfRule type="colorScale" priority="320">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H18 J18 D18:F18">
-    <cfRule type="colorScale" priority="319">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H21 J21 D21 F21">
-    <cfRule type="colorScale" priority="316">
+  <conditionalFormatting sqref="H15 J15 D15 F15">
+    <cfRule type="colorScale" priority="322">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19 J19 D19 F19">
+    <cfRule type="colorScale" priority="318">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20 J20 D20:F20">
+    <cfRule type="colorScale" priority="317">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4659,6 +4555,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J5 F5 D5 H5">
+    <cfRule type="colorScale" priority="332">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5">
     <cfRule type="colorScale" priority="368">
       <colorScale>
@@ -4671,6 +4579,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J6 F6 D6 H6">
+    <cfRule type="colorScale" priority="331">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J6">
     <cfRule type="colorScale" priority="367">
       <colorScale>
@@ -4683,6 +4603,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J7 F7 D7 H7">
+    <cfRule type="colorScale" priority="330">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J7">
     <cfRule type="colorScale" priority="366">
       <colorScale>
@@ -4695,6 +4627,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J8 D8 F8 H8">
+    <cfRule type="colorScale" priority="329">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J8">
     <cfRule type="colorScale" priority="365">
       <colorScale>
@@ -4707,6 +4651,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J9 F9 D9 H9">
+    <cfRule type="colorScale" priority="328">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J9">
     <cfRule type="colorScale" priority="364">
       <colorScale>
@@ -4719,6 +4675,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J10 F10 D10 H10">
+    <cfRule type="colorScale" priority="327">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J10">
     <cfRule type="colorScale" priority="363">
       <colorScale>
@@ -4731,18 +4699,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J11 F11 D11 H11">
-    <cfRule type="colorScale" priority="326">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J11">
     <cfRule type="colorScale" priority="362">
       <colorScale>
@@ -4755,18 +4711,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J12 D12 F12 H12">
-    <cfRule type="colorScale" priority="325">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J12">
     <cfRule type="colorScale" priority="361">
       <colorScale>
@@ -4779,6 +4723,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J13 F13 D13 H13">
+    <cfRule type="colorScale" priority="324">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J13">
     <cfRule type="colorScale" priority="360">
       <colorScale>
@@ -4791,6 +4747,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J14 D14 F14 H14">
+    <cfRule type="colorScale" priority="323">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J14">
     <cfRule type="colorScale" priority="359">
       <colorScale>
@@ -4803,18 +4771,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J15 H15 D15 F15">
-    <cfRule type="colorScale" priority="322">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J15">
     <cfRule type="colorScale" priority="358">
       <colorScale>
@@ -4827,6 +4783,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J16 D16 F16 H16">
+    <cfRule type="colorScale" priority="321">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J16">
     <cfRule type="colorScale" priority="357">
       <colorScale>
@@ -4839,6 +4807,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J17 H17 D17 F17">
+    <cfRule type="colorScale" priority="320">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J17">
     <cfRule type="colorScale" priority="356">
       <colorScale>
@@ -4851,6 +4831,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J18 H18 D18:F18">
+    <cfRule type="colorScale" priority="319">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J18">
     <cfRule type="colorScale" priority="355">
       <colorScale>
@@ -4863,18 +4855,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J19 H19 D19 F19">
-    <cfRule type="colorScale" priority="318">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J19">
     <cfRule type="colorScale" priority="354">
       <colorScale>
@@ -4887,18 +4867,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J20 H20 D20:F20">
-    <cfRule type="colorScale" priority="317">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J20">
     <cfRule type="colorScale" priority="353">
       <colorScale>
@@ -4911,8 +4879,32 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J21 H21 D21 F21">
+    <cfRule type="colorScale" priority="316">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J21">
     <cfRule type="colorScale" priority="352">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J22 D22 F22 H22">
+    <cfRule type="colorScale" priority="315">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>